<commit_message>
Finalize Assignment 5 financial model deliverables
</commit_message>
<xml_diff>
--- a/railguard_financial_model.xlsx
+++ b/railguard_financial_model.xlsx
@@ -1715,19 +1715,19 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>180000</v>
+        <v>70000</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>320000</v>
+        <v>120000</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>700000</v>
+        <v>220000</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>1400000</v>
+        <v>620000</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>2700000</v>
+        <v>1200000</v>
       </c>
     </row>
     <row r="3">
@@ -1737,19 +1737,19 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>60000</v>
+        <v>35000</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>80000</v>
+        <v>45000</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>110000</v>
+        <v>70000</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>170000</v>
+        <v>120000</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>250000</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="4">
@@ -1759,19 +1759,19 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>20000</v>
+        <v>12000</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>40000</v>
+        <v>18000</v>
       </c>
       <c r="D4" s="2" t="n">
+        <v>35000</v>
+      </c>
+      <c r="E4" s="2" t="n">
         <v>70000</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="F4" s="2" t="n">
         <v>120000</v>
-      </c>
-      <c r="F4" s="2" t="n">
-        <v>180000</v>
       </c>
     </row>
     <row r="5">
@@ -1781,19 +1781,19 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>45000</v>
+        <v>28000</v>
       </c>
       <c r="C5" s="2" t="n">
+        <v>40000</v>
+      </c>
+      <c r="D5" s="2" t="n">
         <v>65000</v>
       </c>
-      <c r="D5" s="2" t="n">
-        <v>95000</v>
-      </c>
       <c r="E5" s="2" t="n">
-        <v>140000</v>
+        <v>130000</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>190000</v>
+        <v>210000</v>
       </c>
     </row>
     <row r="6">
@@ -1803,19 +1803,19 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>40000</v>
+        <v>25000</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>55000</v>
+        <v>45000</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>85000</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>130000</v>
+        <v>180000</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>180000</v>
+        <v>250000</v>
       </c>
     </row>
     <row r="7">
@@ -1825,19 +1825,19 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>23000</v>
+        <v>18000</v>
       </c>
       <c r="C7" s="2" t="n">
         <v>30000</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>45000</v>
+        <v>58000</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>70000</v>
+        <v>98000</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>95000</v>
+        <v>117000</v>
       </c>
     </row>
     <row r="8">
@@ -2304,9 +2304,8 @@
       <c r="B2" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="C2">
-        <f>Opex!B2</f>
-        <v/>
+      <c r="C2" s="2" t="n">
+        <v>180000</v>
       </c>
       <c r="D2">
         <f>C2/B2</f>
@@ -2334,9 +2333,8 @@
       <c r="B3" s="2" t="n">
         <v>230</v>
       </c>
-      <c r="C3">
-        <f>Opex!C2</f>
-        <v/>
+      <c r="C3" s="2" t="n">
+        <v>320000</v>
       </c>
       <c r="D3">
         <f>C3/B3</f>
@@ -2364,9 +2362,8 @@
       <c r="B4" s="2" t="n">
         <v>580</v>
       </c>
-      <c r="C4">
-        <f>Opex!D2</f>
-        <v/>
+      <c r="C4" s="2" t="n">
+        <v>700000</v>
       </c>
       <c r="D4">
         <f>C4/B4</f>
@@ -2394,9 +2391,8 @@
       <c r="B5" s="2" t="n">
         <v>1200</v>
       </c>
-      <c r="C5">
-        <f>Opex!E2</f>
-        <v/>
+      <c r="C5" s="2" t="n">
+        <v>1400000</v>
       </c>
       <c r="D5">
         <f>C5/B5</f>
@@ -2424,9 +2420,8 @@
       <c r="B6" s="2" t="n">
         <v>2100</v>
       </c>
-      <c r="C6">
-        <f>Opex!F2</f>
-        <v/>
+      <c r="C6" s="2" t="n">
+        <v>2700000</v>
       </c>
       <c r="D6">
         <f>C6/B6</f>
@@ -2456,7 +2451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2538,7 +2533,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Marketing spend</t>
+          <t>Marketing spend (non-payroll)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -2550,70 +2545,82 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Payroll assumptions</t>
+          <t>GTM spend for CAC payback</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Hiring!A2:G9 and Hiring!B13:F13</t>
+          <t>CAC_Payback!C2:C6</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Other SG&amp;A</t>
+          <t>Payroll assumptions</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Opex!B8:F8</t>
+          <t>Hiring!A2:G9 and Hiring!B13:F13</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Revenue</t>
+          <t>Other SG&amp;A</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Financials!B2:F2</t>
+          <t>Opex!B8:F8</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Gross margin</t>
+          <t>Revenue</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>COGS!F10:F14</t>
+          <t>Financials!B2:F2</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>EBITDA</t>
+          <t>Gross margin</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Financials!B8:F8</t>
+          <t>COGS!F10:F14</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>EBITDA</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Financials!B8:F8</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>Cash flow and cash balance</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>Financials!B11:F13</t>
         </is>

</xml_diff>